<commit_message>
2nd vs 4th suspense
</commit_message>
<xml_diff>
--- a/data/out/wiki/men/uefa/eu/goals_eu_uefa.xlsx
+++ b/data/out/wiki/men/uefa/eu/goals_eu_uefa.xlsx
@@ -678,7 +678,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>['Denmark', 'France']</t>
+          <t>['France', 'Denmark']</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2398,7 +2398,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>['Spain', 'West Germany']</t>
+          <t>['West Germany', 'Spain']</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -5644,7 +5644,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>['Germany', 'Netherlands']</t>
+          <t>['Netherlands', 'Germany']</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -8136,7 +8136,7 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>['Netherlands', 'England']</t>
+          <t>['England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>['Netherlands', 'England']</t>
+          <t>['England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -8448,7 +8448,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>['Netherlands', 'England']</t>
+          <t>['England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>['Netherlands', 'England']</t>
+          <t>['England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>['Netherlands', 'England']</t>
+          <t>['England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>['England', 'Scotland']</t>
+          <t>['Scotland', 'England']</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>['Netherlands', 'England']</t>
+          <t>['England', 'Netherlands']</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>['Croatia', 'Portugal']</t>
+          <t>['Portugal', 'Croatia']</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -9536,7 +9536,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>['Croatia', 'Portugal']</t>
+          <t>['Portugal', 'Croatia']</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -9694,7 +9694,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>['Croatia', 'Portugal']</t>
+          <t>['Portugal', 'Croatia']</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -9852,7 +9852,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>['Croatia', 'Portugal']</t>
+          <t>['Portugal', 'Croatia']</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>['Croatia', 'Portugal']</t>
+          <t>['Portugal', 'Croatia']</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>['Croatia', 'Portugal']</t>
+          <t>['Portugal', 'Croatia']</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -10312,7 +10312,7 @@
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -10624,7 +10624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -10940,7 +10940,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -11098,7 +11098,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>['Germany', 'Italy']</t>
+          <t>['Italy', 'Germany']</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -11211,7 +11211,7 @@
         <v>0</v>
       </c>
       <c r="AR69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -11256,7 +11256,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -11400,7 +11400,7 @@
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>['Belgium', 'Italy']</t>
+          <t>['Italy', 'Belgium']</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>['Belgium', 'Italy']</t>
+          <t>['Italy', 'Belgium']</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>['Turkey', 'Italy']</t>
+          <t>['Italy', 'Turkey']</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>['Turkey', 'Italy']</t>
+          <t>['Italy', 'Turkey']</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -12028,7 +12028,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>['Turkey', 'Italy']</t>
+          <t>['Italy', 'Turkey']</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -12186,7 +12186,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>['Turkey', 'Italy']</t>
+          <t>['Italy', 'Turkey']</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -12330,7 +12330,7 @@
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
-          <t>['England', 'Portugal']</t>
+          <t>['Portugal', 'England']</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -12484,7 +12484,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>['Romania', 'Portugal']</t>
+          <t>['Portugal', 'Romania']</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -12642,7 +12642,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>['Romania', 'Portugal']</t>
+          <t>['Portugal', 'Romania']</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -12800,7 +12800,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>['England', 'Portugal']</t>
+          <t>['Portugal', 'England']</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>['England', 'Portugal']</t>
+          <t>['Portugal', 'England']</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>['England', 'Portugal']</t>
+          <t>['Portugal', 'England']</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -13274,7 +13274,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>['England', 'Portugal']</t>
+          <t>['Portugal', 'England']</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -13432,7 +13432,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>['England', 'Portugal']</t>
+          <t>['Portugal', 'England']</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -13590,7 +13590,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>['Romania', 'Portugal']</t>
+          <t>['Portugal', 'Romania']</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -13734,7 +13734,7 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -13888,7 +13888,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -14362,7 +14362,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -14678,7 +14678,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>['Norway', 'Yugoslavia']</t>
+          <t>['Yugoslavia', 'Norway']</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -14980,7 +14980,7 @@
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -15134,7 +15134,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -15450,7 +15450,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -15608,7 +15608,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -15766,7 +15766,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -15924,7 +15924,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -16082,7 +16082,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France']</t>
+          <t>['France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -16854,7 +16854,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>['Greece', 'Portugal']</t>
+          <t>['Portugal', 'Greece']</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -16998,7 +16998,7 @@
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -17626,7 +17626,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -17784,7 +17784,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -17942,7 +17942,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -18100,7 +18100,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -18258,7 +18258,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -18416,7 +18416,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -18574,7 +18574,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -19964,7 +19964,7 @@
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -20118,7 +20118,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -20276,7 +20276,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>['Germany', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Germany']</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -20434,7 +20434,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -20592,7 +20592,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -20750,7 +20750,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -21052,7 +21052,7 @@
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -21206,7 +21206,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -21364,7 +21364,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -21522,7 +21522,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -21680,7 +21680,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -21838,7 +21838,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -21996,7 +21996,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -22154,7 +22154,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>['Turkey', 'Portugal']</t>
+          <t>['Portugal', 'Turkey']</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -22298,7 +22298,7 @@
       <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr">
         <is>
-          <t>['Germany', 'Croatia']</t>
+          <t>['Croatia', 'Germany']</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -22452,7 +22452,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>['Germany', 'Croatia']</t>
+          <t>['Croatia', 'Germany']</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -22610,7 +22610,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>['Germany', 'Croatia']</t>
+          <t>['Croatia', 'Germany']</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -22908,7 +22908,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Italy']</t>
+          <t>['Italy', 'Netherlands']</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -23066,7 +23066,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Italy']</t>
+          <t>['Italy', 'Netherlands']</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -23224,7 +23224,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Italy']</t>
+          <t>['Italy', 'Netherlands']</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -23382,7 +23382,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Italy']</t>
+          <t>['Italy', 'Netherlands']</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -23526,7 +23526,7 @@
       <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
-          <t>['Spain', 'Sweden']</t>
+          <t>['Sweden', 'Spain']</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -24456,7 +24456,7 @@
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Russia']</t>
+          <t>['Russia', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -24610,7 +24610,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>['Greece', 'Russia']</t>
+          <t>['Russia', 'Greece']</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -24768,7 +24768,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Greece']</t>
+          <t>['Greece', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -24912,7 +24912,7 @@
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr">
         <is>
-          <t>['Germany', 'Portugal']</t>
+          <t>['Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -25066,7 +25066,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>['Germany', 'Denmark']</t>
+          <t>['Denmark', 'Germany']</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -25224,7 +25224,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>['Germany', 'Portugal']</t>
+          <t>['Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -25382,7 +25382,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>['Germany', 'Denmark']</t>
+          <t>['Denmark', 'Germany']</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -25540,7 +25540,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>['Germany', 'Portugal']</t>
+          <t>['Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -25698,7 +25698,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>['Germany', 'Portugal']</t>
+          <t>['Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -25856,7 +25856,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>['Germany', 'Portugal']</t>
+          <t>['Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -26614,7 +26614,7 @@
       <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -26768,7 +26768,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -26926,7 +26926,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -27084,7 +27084,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>['England', 'France']</t>
+          <t>['France', 'England']</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -27228,7 +27228,7 @@
       <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Romania', 'France']</t>
+          <t>['France', 'Switzerland', 'Romania']</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -27382,7 +27382,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>['Switzerland', 'France', 'Albania']</t>
+          <t>['France', 'Switzerland', 'Albania']</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -27526,7 +27526,7 @@
       <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr">
         <is>
-          <t>['England', 'Wales', 'Slovakia']</t>
+          <t>['Slovakia', 'England', 'Wales']</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -27680,7 +27680,7 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>['England', 'Wales', 'Slovakia']</t>
+          <t>['Slovakia', 'England', 'Wales']</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -27838,7 +27838,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>['England', 'Wales', 'Slovakia']</t>
+          <t>['Slovakia', 'England', 'Wales']</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -27996,7 +27996,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>['England', 'Wales', 'Slovakia']</t>
+          <t>['Slovakia', 'England', 'Wales']</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -28140,7 +28140,7 @@
       <c r="I179" t="inlineStr"/>
       <c r="J179" t="inlineStr">
         <is>
-          <t>['Germany', 'Poland', 'Northern Ireland']</t>
+          <t>['Poland', 'Northern Ireland', 'Germany']</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -28294,7 +28294,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>['Germany', 'Poland', 'Northern Ireland']</t>
+          <t>['Poland', 'Northern Ireland', 'Germany']</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -28452,7 +28452,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>['Germany', 'Poland', 'Northern Ireland']</t>
+          <t>['Poland', 'Northern Ireland', 'Germany']</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -28596,7 +28596,7 @@
       <c r="I182" t="inlineStr"/>
       <c r="J182" t="inlineStr">
         <is>
-          <t>['Croatia', 'Czech Republic', 'Spain']</t>
+          <t>['Czech Republic', 'Croatia', 'Spain']</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -28750,7 +28750,7 @@
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>['Croatia', 'Czech Republic', 'Spain']</t>
+          <t>['Czech Republic', 'Croatia', 'Spain']</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -29382,7 +29382,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>['Spain', 'Turkey', 'Croatia']</t>
+          <t>['Turkey', 'Croatia', 'Spain']</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -29526,7 +29526,7 @@
       <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -29680,7 +29680,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -29838,7 +29838,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -29996,7 +29996,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -30154,7 +30154,7 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -30312,7 +30312,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -30470,7 +30470,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -30628,7 +30628,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -30786,7 +30786,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -30944,7 +30944,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>['Iceland', 'Portugal', 'Hungary']</t>
+          <t>['Hungary', 'Iceland', 'Portugal']</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -31088,7 +31088,7 @@
       <c r="I198" t="inlineStr"/>
       <c r="J198" t="inlineStr">
         <is>
-          <t>['Belgium', 'Italy', 'Sweden']</t>
+          <t>['Italy', 'Belgium', 'Sweden']</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -31242,7 +31242,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>['Ireland', 'Belgium', 'Italy']</t>
+          <t>['Italy', 'Ireland', 'Belgium']</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -31400,7 +31400,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>['Ireland', 'Belgium', 'Italy']</t>
+          <t>['Italy', 'Ireland', 'Belgium']</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -31544,7 +31544,7 @@
       <c r="I201" t="inlineStr"/>
       <c r="J201" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Wales', 'Italy']</t>
+          <t>['Italy', 'Wales', 'Switzerland']</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -31698,7 +31698,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Wales', 'Italy']</t>
+          <t>['Italy', 'Wales', 'Switzerland']</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -31856,7 +31856,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Wales', 'Italy']</t>
+          <t>['Italy', 'Wales', 'Switzerland']</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -32014,7 +32014,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Wales', 'Italy']</t>
+          <t>['Italy', 'Wales', 'Switzerland']</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -32172,7 +32172,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Wales', 'Italy']</t>
+          <t>['Italy', 'Wales', 'Switzerland']</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -32330,7 +32330,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Wales', 'Italy']</t>
+          <t>['Italy', 'Wales', 'Switzerland']</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -32474,7 +32474,7 @@
       <c r="I207" t="inlineStr"/>
       <c r="J207" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Austria', 'Ukraine', 'Netherlands']</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -32628,7 +32628,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Austria', 'Ukraine', 'Netherlands']</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -32786,7 +32786,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Austria', 'Ukraine', 'Netherlands']</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -32944,7 +32944,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Austria', 'Ukraine', 'Netherlands']</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -33102,7 +33102,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Austria', 'Ukraine', 'Netherlands']</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -33400,7 +33400,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Finland']</t>
+          <t>['Belgium', 'Finland', 'Denmark']</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -33558,7 +33558,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Finland']</t>
+          <t>['Belgium', 'Finland', 'Denmark']</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -33716,7 +33716,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Finland']</t>
+          <t>['Belgium', 'Finland', 'Denmark']</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -33874,7 +33874,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Russia']</t>
+          <t>['Belgium', 'Russia', 'Denmark']</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -34032,7 +34032,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Finland']</t>
+          <t>['Belgium', 'Finland', 'Denmark']</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -34190,7 +34190,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Finland']</t>
+          <t>['Belgium', 'Finland', 'Denmark']</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -34348,7 +34348,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>['Denmark', 'Belgium', 'Finland']</t>
+          <t>['Belgium', 'Finland', 'Denmark']</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -34492,7 +34492,7 @@
       <c r="I220" t="inlineStr"/>
       <c r="J220" t="inlineStr">
         <is>
-          <t>['England', 'Czech Republic', 'Croatia']</t>
+          <t>['Czech Republic', 'England', 'Croatia']</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -34646,7 +34646,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>['England', 'Czech Republic', 'Croatia']</t>
+          <t>['Czech Republic', 'England', 'Croatia']</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -34804,7 +34804,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>['England', 'Czech Republic', 'Croatia']</t>
+          <t>['Czech Republic', 'England', 'Croatia']</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -34962,7 +34962,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>['England', 'Czech Republic', 'Croatia']</t>
+          <t>['Czech Republic', 'England', 'Croatia']</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -35120,7 +35120,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>['England', 'Czech Republic', 'Croatia']</t>
+          <t>['Czech Republic', 'England', 'Croatia']</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -35278,7 +35278,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>['England', 'Czech Republic', 'Croatia']</t>
+          <t>['Czech Republic', 'England', 'Croatia']</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -35422,7 +35422,7 @@
       <c r="I226" t="inlineStr"/>
       <c r="J226" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -35576,7 +35576,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -35734,7 +35734,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -35892,7 +35892,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -36050,7 +36050,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -36208,7 +36208,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -36366,7 +36366,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -36524,7 +36524,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -36682,7 +36682,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -36840,7 +36840,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Sweden', 'Slovakia', 'Spain']</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -36998,7 +36998,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>['Slovakia', 'Spain', 'Sweden']</t>
+          <t>['Spain', 'Slovakia', 'Sweden']</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -37142,7 +37142,7 @@
       <c r="I237" t="inlineStr"/>
       <c r="J237" t="inlineStr">
         <is>
-          <t>['Germany', 'France', 'Portugal']</t>
+          <t>['France', 'Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -37770,7 +37770,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>['Germany', 'France', 'Hungary']</t>
+          <t>['France', 'Hungary', 'Germany']</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -38086,7 +38086,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>['Germany', 'France', 'Portugal']</t>
+          <t>['France', 'Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -38402,7 +38402,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>['Germany', 'France', 'Portugal']</t>
+          <t>['France', 'Portugal', 'Germany']</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -38546,7 +38546,7 @@
       <c r="I246" t="inlineStr"/>
       <c r="J246" t="inlineStr">
         <is>
-          <t>['Germany', 'Switzerland', 'Scotland']</t>
+          <t>['Scotland', 'Switzerland', 'Germany']</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -38700,7 +38700,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>['Switzerland', 'Germany', 'Scotland']</t>
+          <t>['Scotland', 'Switzerland', 'Germany']</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -38858,7 +38858,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>['Germany', 'Switzerland', 'Scotland']</t>
+          <t>['Scotland', 'Switzerland', 'Germany']</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -39016,7 +39016,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>['Germany', 'Switzerland', 'Hungary']</t>
+          <t>['Hungary', 'Switzerland', 'Germany']</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -39160,7 +39160,7 @@
       <c r="I250" t="inlineStr"/>
       <c r="J250" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain', 'Albania']</t>
+          <t>['Italy', 'Albania', 'Spain']</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -39314,7 +39314,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>['Croatia', 'Italy', 'Spain']</t>
+          <t>['Italy', 'Croatia', 'Spain']</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -39472,7 +39472,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>['Croatia', 'Italy', 'Spain']</t>
+          <t>['Italy', 'Croatia', 'Spain']</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -39630,7 +39630,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>['Croatia', 'Italy', 'Spain']</t>
+          <t>['Italy', 'Croatia', 'Spain']</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -39774,7 +39774,7 @@
       <c r="I254" t="inlineStr"/>
       <c r="J254" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Austria', 'France']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -39928,7 +39928,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -40086,7 +40086,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Austria', 'France']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -40244,7 +40244,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Austria', 'France']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -40402,7 +40402,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Austria', 'France']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -40560,7 +40560,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Austria', 'France']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -40718,7 +40718,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Austria', 'France']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -40876,7 +40876,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>['Netherlands', 'France', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -41160,7 +41160,7 @@
       <c r="I263" t="inlineStr"/>
       <c r="J263" t="inlineStr">
         <is>
-          <t>['Romania', 'Belgium', 'Slovakia']</t>
+          <t>['Belgium', 'Slovakia', 'Romania']</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -41314,7 +41314,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>['Ukraine', 'Belgium', 'Slovakia']</t>
+          <t>['Belgium', 'Ukraine', 'Slovakia']</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -41472,7 +41472,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>['Romania', 'Belgium', 'Slovakia']</t>
+          <t>['Belgium', 'Slovakia', 'Romania']</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -41616,7 +41616,7 @@
       <c r="I266" t="inlineStr"/>
       <c r="J266" t="inlineStr">
         <is>
-          <t>['Turkey', 'Czech Republic', 'Portugal']</t>
+          <t>['Portugal', 'Czech Republic', 'Turkey']</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -41770,7 +41770,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>['Turkey', 'Georgia', 'Portugal']</t>
+          <t>['Portugal', 'Turkey', 'Georgia']</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -41928,7 +41928,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>['Turkey', 'Georgia', 'Portugal']</t>
+          <t>['Portugal', 'Turkey', 'Georgia']</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -42086,7 +42086,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>['Turkey', 'Georgia', 'Portugal']</t>
+          <t>['Portugal', 'Turkey', 'Georgia']</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -42244,7 +42244,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>['Turkey', 'Georgia', 'Portugal']</t>
+          <t>['Portugal', 'Turkey', 'Georgia']</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -42402,7 +42402,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>['Turkey', 'Georgia', 'Portugal']</t>
+          <t>['Portugal', 'Turkey', 'Georgia']</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">

</xml_diff>

<commit_message>
2nd and 4th eu uefa
</commit_message>
<xml_diff>
--- a/data/out/wiki/men/uefa/eu/goals_eu_uefa.xlsx
+++ b/data/out/wiki/men/uefa/eu/goals_eu_uefa.xlsx
@@ -678,7 +678,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>['France', 'Denmark']</t>
+          <t>['Denmark', 'France']</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>['France', 'Belgium']</t>
+          <t>['Belgium', 'France']</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>['France', 'Belgium']</t>
+          <t>['Belgium', 'France']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>['France', 'Belgium']</t>
+          <t>['Belgium', 'France']</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>['France', 'Belgium']</t>
+          <t>['Belgium', 'France']</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>['France', 'Belgium']</t>
+          <t>['Belgium', 'France']</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>['France', 'Denmark']</t>
+          <t>['Denmark', 'France']</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>['France', 'Denmark']</t>
+          <t>['Denmark', 'France']</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>['France', 'Denmark']</t>
+          <t>['Denmark', 'France']</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>['France', 'Denmark']</t>
+          <t>['Denmark', 'France']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>['France', 'Denmark']</t>
+          <t>['Denmark', 'France']</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2398,7 +2398,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>['West Germany', 'Spain']</t>
+          <t>['Spain', 'West Germany']</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>['Portugal', 'Spain']</t>
+          <t>['Spain', 'Portugal']</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Soviet Union']</t>
+          <t>['Soviet Union', 'Netherlands']</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -5644,7 +5644,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Germany']</t>
+          <t>['Germany', 'Netherlands']</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>['France', 'Spain']</t>
+          <t>['Spain', 'France']</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>['France', 'Spain']</t>
+          <t>['Spain', 'France']</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>['France', 'Spain']</t>
+          <t>['Spain', 'France']</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>['Italy', 'Turkey']</t>
+          <t>['Turkey', 'Italy']</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>['Italy', 'Turkey']</t>
+          <t>['Turkey', 'Italy']</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -12028,7 +12028,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>['Italy', 'Turkey']</t>
+          <t>['Turkey', 'Italy']</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -12186,7 +12186,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>['Italy', 'Turkey']</t>
+          <t>['Turkey', 'Italy']</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -13734,7 +13734,7 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -13888,7 +13888,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -14362,7 +14362,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -14678,7 +14678,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Norway']</t>
+          <t>['Norway', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -14836,7 +14836,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>['Yugoslavia', 'Spain']</t>
+          <t>['Spain', 'Yugoslavia']</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -16854,7 +16854,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>['Portugal', 'Greece']</t>
+          <t>['Greece', 'Portugal']</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -17152,7 +17152,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>['France', 'Croatia']</t>
+          <t>['Croatia', 'France']</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -17310,7 +17310,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>['France', 'Croatia']</t>
+          <t>['Croatia', 'France']</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -17468,7 +17468,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>['France', 'Croatia']</t>
+          <t>['Croatia', 'France']</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -18718,7 +18718,7 @@
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -18872,7 +18872,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -19030,7 +19030,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -19188,7 +19188,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -19346,7 +19346,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -19504,7 +19504,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -19662,7 +19662,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -19820,7 +19820,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>['Sweden', 'Denmark']</t>
+          <t>['Denmark', 'Sweden']</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -20434,7 +20434,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -20592,7 +20592,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -20750,7 +20750,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -20908,7 +20908,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Czech Republic']</t>
+          <t>['Czech Republic', 'Netherlands']</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -22754,7 +22754,7 @@
       <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Romania']</t>
+          <t>['Romania', 'Netherlands']</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -23526,7 +23526,7 @@
       <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain']</t>
+          <t>['Spain', 'Sweden']</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -24610,7 +24610,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>['Russia', 'Greece']</t>
+          <t>['Greece', 'Russia']</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -24768,7 +24768,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>['Czech Republic', 'Greece']</t>
+          <t>['Greece', 'Czech Republic']</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -26154,7 +26154,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain']</t>
+          <t>['Spain', 'Italy']</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -26312,7 +26312,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain']</t>
+          <t>['Spain', 'Italy']</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -26470,7 +26470,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain']</t>
+          <t>['Spain', 'Italy']</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -27228,7 +27228,7 @@
       <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr">
         <is>
-          <t>['France', 'Switzerland', 'Romania']</t>
+          <t>['Switzerland', 'France', 'Romania']</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -27382,7 +27382,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>['France', 'Albania', 'Switzerland']</t>
+          <t>['Albania', 'Switzerland', 'France']</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -28140,7 +28140,7 @@
       <c r="I179" t="inlineStr"/>
       <c r="J179" t="inlineStr">
         <is>
-          <t>['Poland', 'Northern Ireland', 'Germany']</t>
+          <t>['Northern Ireland', 'Poland', 'Germany']</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -28294,7 +28294,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>['Poland', 'Northern Ireland', 'Germany']</t>
+          <t>['Northern Ireland', 'Poland', 'Germany']</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -28452,7 +28452,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>['Poland', 'Northern Ireland', 'Germany']</t>
+          <t>['Northern Ireland', 'Poland', 'Germany']</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -28908,7 +28908,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>['Spain', 'Turkey', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Turkey']</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -29066,7 +29066,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>['Spain', 'Turkey', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Turkey']</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -29224,7 +29224,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>['Spain', 'Turkey', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Turkey']</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -29382,7 +29382,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>['Spain', 'Turkey', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Turkey']</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -29526,7 +29526,7 @@
       <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -29680,7 +29680,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -29838,7 +29838,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -29996,7 +29996,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -30154,7 +30154,7 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -30312,7 +30312,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -30470,7 +30470,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -30628,7 +30628,7 @@
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -30786,7 +30786,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -30944,7 +30944,7 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'Iceland']</t>
+          <t>['Portugal', 'Iceland', 'Hungary']</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -31242,7 +31242,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>['Ireland', 'Belgium', 'Italy']</t>
+          <t>['Belgium', 'Ireland', 'Italy']</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -31400,7 +31400,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>['Ireland', 'Belgium', 'Italy']</t>
+          <t>['Belgium', 'Ireland', 'Italy']</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -31544,7 +31544,7 @@
       <c r="I201" t="inlineStr"/>
       <c r="J201" t="inlineStr">
         <is>
-          <t>['Wales', 'Italy', 'Switzerland']</t>
+          <t>['Wales', 'Switzerland', 'Italy']</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -31698,7 +31698,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>['Wales', 'Italy', 'Switzerland']</t>
+          <t>['Wales', 'Switzerland', 'Italy']</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -31856,7 +31856,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>['Wales', 'Italy', 'Switzerland']</t>
+          <t>['Wales', 'Switzerland', 'Italy']</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -32014,7 +32014,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>['Wales', 'Italy', 'Switzerland']</t>
+          <t>['Wales', 'Switzerland', 'Italy']</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -32172,7 +32172,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>['Wales', 'Italy', 'Switzerland']</t>
+          <t>['Wales', 'Switzerland', 'Italy']</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -32330,7 +32330,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>['Wales', 'Italy', 'Switzerland']</t>
+          <t>['Wales', 'Switzerland', 'Italy']</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -32474,7 +32474,7 @@
       <c r="I207" t="inlineStr"/>
       <c r="J207" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Ukraine', 'Austria', 'Netherlands']</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -32628,7 +32628,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Ukraine', 'Austria', 'Netherlands']</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -32786,7 +32786,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Ukraine', 'Austria', 'Netherlands']</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -32944,7 +32944,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Ukraine', 'Austria', 'Netherlands']</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -33102,7 +33102,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>['Netherlands', 'Ukraine', 'Austria']</t>
+          <t>['Ukraine', 'Austria', 'Netherlands']</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -33874,7 +33874,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>['Belgium', 'Russia', 'Denmark']</t>
+          <t>['Russia', 'Belgium', 'Denmark']</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -35422,7 +35422,7 @@
       <c r="I226" t="inlineStr"/>
       <c r="J226" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -35576,7 +35576,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -35734,7 +35734,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -35892,7 +35892,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -36050,7 +36050,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -36208,7 +36208,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -36366,7 +36366,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -36524,7 +36524,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -36682,7 +36682,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -36840,7 +36840,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -36998,7 +36998,7 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>['Sweden', 'Spain', 'Slovakia']</t>
+          <t>['Spain', 'Sweden', 'Slovakia']</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -37142,7 +37142,7 @@
       <c r="I237" t="inlineStr"/>
       <c r="J237" t="inlineStr">
         <is>
-          <t>['France', 'Portugal', 'Germany']</t>
+          <t>['Portugal', 'France', 'Germany']</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -37296,7 +37296,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>['France', 'Hungary', 'Portugal']</t>
+          <t>['Portugal', 'France', 'Hungary']</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -37454,7 +37454,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>['Portugal', 'Hungary', 'France']</t>
+          <t>['Portugal', 'France', 'Hungary']</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -37612,7 +37612,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>['France', 'Hungary', 'Portugal']</t>
+          <t>['Portugal', 'France', 'Hungary']</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -37928,7 +37928,7 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>['France', 'Hungary', 'Portugal']</t>
+          <t>['Portugal', 'France', 'Hungary']</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -38086,7 +38086,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>['France', 'Portugal', 'Germany']</t>
+          <t>['Portugal', 'France', 'Germany']</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -38244,7 +38244,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>['France', 'Hungary', 'Portugal']</t>
+          <t>['Portugal', 'France', 'Hungary']</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -38402,7 +38402,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>['France', 'Portugal', 'Germany']</t>
+          <t>['Portugal', 'France', 'Germany']</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -39160,7 +39160,7 @@
       <c r="I250" t="inlineStr"/>
       <c r="J250" t="inlineStr">
         <is>
-          <t>['Italy', 'Albania', 'Spain']</t>
+          <t>['Spain', 'Italy', 'Albania']</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -39314,7 +39314,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Italy']</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -39472,7 +39472,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Italy']</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -39630,7 +39630,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>['Italy', 'Spain', 'Croatia']</t>
+          <t>['Spain', 'Croatia', 'Italy']</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -39774,7 +39774,7 @@
       <c r="I254" t="inlineStr"/>
       <c r="J254" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -39928,7 +39928,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -40086,7 +40086,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -40244,7 +40244,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -40402,7 +40402,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -40560,7 +40560,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -40718,7 +40718,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -40876,7 +40876,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>['France', 'Netherlands', 'Austria']</t>
+          <t>['Austria', 'France', 'Netherlands']</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -41314,7 +41314,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>['Belgium', 'Ukraine', 'Slovakia']</t>
+          <t>['Ukraine', 'Belgium', 'Slovakia']</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -41770,7 +41770,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>['Portugal', 'Georgia', 'Turkey']</t>
+          <t>['Georgia', 'Portugal', 'Turkey']</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -41928,7 +41928,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>['Portugal', 'Georgia', 'Turkey']</t>
+          <t>['Georgia', 'Portugal', 'Turkey']</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -42086,7 +42086,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>['Portugal', 'Georgia', 'Turkey']</t>
+          <t>['Georgia', 'Portugal', 'Turkey']</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -42244,7 +42244,7 @@
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>['Portugal', 'Georgia', 'Turkey']</t>
+          <t>['Georgia', 'Portugal', 'Turkey']</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -42402,7 +42402,7 @@
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>['Portugal', 'Georgia', 'Turkey']</t>
+          <t>['Georgia', 'Portugal', 'Turkey']</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">

</xml_diff>